<commit_message>
feat: standardize RunnerX on English-only content
</commit_message>
<xml_diff>
--- a/data/sample/registrations.xlsx
+++ b/data/sample/registrations.xlsx
@@ -137,286 +137,286 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
+<ns0:theme xmlns:ns0="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <ns0:themeElements>
+    <ns0:clrScheme name="Office">
+      <ns0:dk1>
+        <ns0:sysClr val="windowText" lastClr="000000"/>
+      </ns0:dk1>
+      <ns0:lt1>
+        <ns0:sysClr val="window" lastClr="FFFFFF"/>
+      </ns0:lt1>
+      <ns0:dk2>
+        <ns0:srgbClr val="1F497D"/>
+      </ns0:dk2>
+      <ns0:lt2>
+        <ns0:srgbClr val="EEECE1"/>
+      </ns0:lt2>
+      <ns0:accent1>
+        <ns0:srgbClr val="4F81BD"/>
+      </ns0:accent1>
+      <ns0:accent2>
+        <ns0:srgbClr val="C0504D"/>
+      </ns0:accent2>
+      <ns0:accent3>
+        <ns0:srgbClr val="9BBB59"/>
+      </ns0:accent3>
+      <ns0:accent4>
+        <ns0:srgbClr val="8064A2"/>
+      </ns0:accent4>
+      <ns0:accent5>
+        <ns0:srgbClr val="4BACC6"/>
+      </ns0:accent5>
+      <ns0:accent6>
+        <ns0:srgbClr val="F79646"/>
+      </ns0:accent6>
+      <ns0:hlink>
+        <ns0:srgbClr val="0000FF"/>
+      </ns0:hlink>
+      <ns0:folHlink>
+        <ns0:srgbClr val="800080"/>
+      </ns0:folHlink>
+    </ns0:clrScheme>
+    <ns0:fontScheme name="Office">
+      <ns0:majorFont>
+        <ns0:latin typeface="Cambria"/>
+        <ns0:ea typeface=""/>
+        <ns0:cs typeface=""/>
+        <ns0:font script="Jpan" typeface="Calibri"/>
+        <ns0:font script="Hang" typeface="Calibri"/>
+        <ns0:font script="Hans" typeface="Calibri"/>
+        <ns0:font script="Hant" typeface="Calibri"/>
+        <ns0:font script="Arab" typeface="Times New Roman"/>
+        <ns0:font script="Hebr" typeface="Times New Roman"/>
+        <ns0:font script="Thai" typeface="Tahoma"/>
+        <ns0:font script="Ethi" typeface="Nyala"/>
+        <ns0:font script="Beng" typeface="Vrinda"/>
+        <ns0:font script="Gujr" typeface="Shruti"/>
+        <ns0:font script="Khmr" typeface="MoolBoran"/>
+        <ns0:font script="Knda" typeface="Tunga"/>
+        <ns0:font script="Guru" typeface="Raavi"/>
+        <ns0:font script="Cans" typeface="Euphemia"/>
+        <ns0:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <ns0:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <ns0:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <ns0:font script="Thaa" typeface="MV Boli"/>
+        <ns0:font script="Deva" typeface="Mangal"/>
+        <ns0:font script="Telu" typeface="Gautami"/>
+        <ns0:font script="Taml" typeface="Latha"/>
+        <ns0:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <ns0:font script="Orya" typeface="Kalinga"/>
+        <ns0:font script="Mlym" typeface="Kartika"/>
+        <ns0:font script="Laoo" typeface="DokChampa"/>
+        <ns0:font script="Sinh" typeface="Iskoola Pota"/>
+        <ns0:font script="Mong" typeface="Mongolian Baiti"/>
+        <ns0:font script="Viet" typeface="Times New Roman"/>
+        <ns0:font script="Uigh" typeface="Microsoft Uighur"/>
+      </ns0:majorFont>
+      <ns0:minorFont>
+        <ns0:latin typeface="Calibri"/>
+        <ns0:ea typeface=""/>
+        <ns0:cs typeface=""/>
+        <ns0:font script="Jpan" typeface="Calibri"/>
+        <ns0:font script="Hang" typeface="Calibri"/>
+        <ns0:font script="Hans" typeface="Calibri"/>
+        <ns0:font script="Hant" typeface="Calibri"/>
+        <ns0:font script="Arab" typeface="Arial"/>
+        <ns0:font script="Hebr" typeface="Arial"/>
+        <ns0:font script="Thai" typeface="Tahoma"/>
+        <ns0:font script="Ethi" typeface="Nyala"/>
+        <ns0:font script="Beng" typeface="Vrinda"/>
+        <ns0:font script="Gujr" typeface="Shruti"/>
+        <ns0:font script="Khmr" typeface="DaunPenh"/>
+        <ns0:font script="Knda" typeface="Tunga"/>
+        <ns0:font script="Guru" typeface="Raavi"/>
+        <ns0:font script="Cans" typeface="Euphemia"/>
+        <ns0:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <ns0:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <ns0:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <ns0:font script="Thaa" typeface="MV Boli"/>
+        <ns0:font script="Deva" typeface="Mangal"/>
+        <ns0:font script="Telu" typeface="Gautami"/>
+        <ns0:font script="Taml" typeface="Latha"/>
+        <ns0:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <ns0:font script="Orya" typeface="Kalinga"/>
+        <ns0:font script="Mlym" typeface="Kartika"/>
+        <ns0:font script="Laoo" typeface="DokChampa"/>
+        <ns0:font script="Sinh" typeface="Iskoola Pota"/>
+        <ns0:font script="Mong" typeface="Mongolian Baiti"/>
+        <ns0:font script="Viet" typeface="Arial"/>
+        <ns0:font script="Uigh" typeface="Microsoft Uighur"/>
+      </ns0:minorFont>
+    </ns0:fontScheme>
+    <ns0:fmtScheme name="Office">
+      <ns0:fillStyleLst>
+        <ns0:solidFill>
+          <ns0:schemeClr val="phClr"/>
+        </ns0:solidFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="50000"/>
+                <ns0:satMod val="300000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="35000">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="37000"/>
+                <ns0:satMod val="300000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="15000"/>
+                <ns0:satMod val="350000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:lin ang="16200000" scaled="1"/>
+        </ns0:gradFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="51000"/>
+                <ns0:satMod val="130000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="80000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="93000"/>
+                <ns0:satMod val="130000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="94000"/>
+                <ns0:satMod val="135000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:lin ang="16200000" scaled="0"/>
+        </ns0:gradFill>
+      </ns0:fillStyleLst>
+      <ns0:lnStyleLst>
+        <ns0:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <ns0:solidFill>
+            <ns0:schemeClr val="phClr">
+              <ns0:shade val="95000"/>
+              <ns0:satMod val="105000"/>
+            </ns0:schemeClr>
+          </ns0:solidFill>
+          <ns0:prstDash val="solid"/>
+        </ns0:ln>
+        <ns0:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <ns0:solidFill>
+            <ns0:schemeClr val="phClr"/>
+          </ns0:solidFill>
+          <ns0:prstDash val="solid"/>
+        </ns0:ln>
+        <ns0:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <ns0:solidFill>
+            <ns0:schemeClr val="phClr"/>
+          </ns0:solidFill>
+          <ns0:prstDash val="solid"/>
+        </ns0:ln>
+      </ns0:lnStyleLst>
+      <ns0:effectStyleLst>
+        <ns0:effectStyle>
+          <ns0:effectLst>
+            <ns0:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <ns0:srgbClr val="000000">
+                <ns0:alpha val="38000"/>
+              </ns0:srgbClr>
+            </ns0:outerShdw>
+          </ns0:effectLst>
+        </ns0:effectStyle>
+        <ns0:effectStyle>
+          <ns0:effectLst>
+            <ns0:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <ns0:srgbClr val="000000">
+                <ns0:alpha val="35000"/>
+              </ns0:srgbClr>
+            </ns0:outerShdw>
+          </ns0:effectLst>
+        </ns0:effectStyle>
+        <ns0:effectStyle>
+          <ns0:effectLst>
+            <ns0:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <ns0:srgbClr val="000000">
+                <ns0:alpha val="35000"/>
+              </ns0:srgbClr>
+            </ns0:outerShdw>
+          </ns0:effectLst>
+          <ns0:scene3d>
+            <ns0:camera prst="orthographicFront">
+              <ns0:rot lat="0" lon="0" rev="0"/>
+            </ns0:camera>
+            <ns0:lightRig rig="threePt" dir="t">
+              <ns0:rot lat="0" lon="0" rev="1200000"/>
+            </ns0:lightRig>
+          </ns0:scene3d>
+          <ns0:sp3d>
+            <ns0:bevelT w="63500" h="25400"/>
+          </ns0:sp3d>
+        </ns0:effectStyle>
+      </ns0:effectStyleLst>
+      <ns0:bgFillStyleLst>
+        <ns0:solidFill>
+          <ns0:schemeClr val="phClr"/>
+        </ns0:solidFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="40000"/>
+                <ns0:satMod val="350000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="40000">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="45000"/>
+                <ns0:shade val="99000"/>
+                <ns0:satMod val="350000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="20000"/>
+                <ns0:satMod val="255000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:path path="circle">
+            <ns0:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </ns0:path>
+        </ns0:gradFill>
+        <ns0:gradFill rotWithShape="1">
+          <ns0:gsLst>
+            <ns0:gs pos="0">
+              <ns0:schemeClr val="phClr">
+                <ns0:tint val="80000"/>
+                <ns0:satMod val="300000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+            <ns0:gs pos="100000">
+              <ns0:schemeClr val="phClr">
+                <ns0:shade val="30000"/>
+                <ns0:satMod val="200000"/>
+              </ns0:schemeClr>
+            </ns0:gs>
+          </ns0:gsLst>
+          <ns0:path path="circle">
+            <ns0:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </ns0:path>
+        </ns0:gradFill>
+      </ns0:bgFillStyleLst>
+    </ns0:fmtScheme>
+  </ns0:themeElements>
+  <ns0:objectDefaults/>
+  <ns0:extraClrSchemeLst/>
+</ns0:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -443,52 +443,52 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>跑者编号</t>
+          <t>external_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>姓名</t>
+          <t>full_name</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>性别</t>
+          <t>gender</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>出生年份</t>
+          <t>birth_year</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>身高(cm)</t>
+          <t>height_cm</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>体重(kg)</t>
+          <t>weight_kg</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>10K测试成绩</t>
+          <t>test_10k_sec</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>全马最佳成绩</t>
+          <t>fm_best_sec</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>备赛周期跑量</t>
+          <t>prep_mileage_km</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>经历与计划</t>
+          <t>experience_text</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -524,7 +524,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3小时3分24秒</t>
+          <t>3:03:24</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -549,7 +549,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -568,7 +568,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3小时31分6秒</t>
+          <t>3:31:06</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -593,7 +593,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -612,7 +612,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3小时21分50秒</t>
+          <t>3:21:50</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -637,7 +637,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -656,7 +656,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>4小时12分2秒</t>
+          <t>4:12:02</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -700,7 +700,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3小时57分36秒</t>
+          <t>3:57:36</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>3小时9分16秒</t>
+          <t>3:09:16</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -769,7 +769,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -788,7 +788,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4小时41分21秒</t>
+          <t>4:41:21</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -813,7 +813,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -832,7 +832,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>4小时50分41秒</t>
+          <t>4:50:41</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -857,7 +857,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3小时25分57秒</t>
+          <t>3:25:57</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -901,7 +901,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -920,7 +920,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3小时33分25秒</t>
+          <t>3:33:25</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -945,7 +945,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -964,7 +964,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>3小时31分34秒</t>
+          <t>3:31:34</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -989,7 +989,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1008,7 +1008,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3小时37分59秒</t>
+          <t>3:37:59</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>4小时28分24秒</t>
+          <t>4:28:24</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3小时2分21秒</t>
+          <t>3:02:21</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>4小时0分8秒</t>
+          <t>4:00:08</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>3小时31分36秒</t>
+          <t>3:31:36</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>4小时51分10秒</t>
+          <t>4:51:10</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1272,7 +1272,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>3小时30分40秒</t>
+          <t>3:30:40</t>
         </is>
       </c>
       <c r="I19" t="n">
@@ -1297,7 +1297,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>4小时48分11秒</t>
+          <t>4:48:11</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3小时10分46秒</t>
+          <t>3:10:46</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>4小时25分40秒</t>
+          <t>4:25:40</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1448,7 +1448,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>3小时44分47秒</t>
+          <t>3:44:47</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>3小时6分54秒</t>
+          <t>3:06:54</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>4小时55分41秒</t>
+          <t>4:55:41</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>4小时31分28秒</t>
+          <t>4:31:28</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>3小时44分17秒</t>
+          <t>3:44:17</t>
         </is>
       </c>
       <c r="I27" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4小时2分46秒</t>
+          <t>4:02:46</t>
         </is>
       </c>
       <c r="I28" t="n">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4小时16分58秒</t>
+          <t>4:16:58</t>
         </is>
       </c>
       <c r="I29" t="n">
@@ -1737,7 +1737,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>M</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>3小时38分37秒</t>
+          <t>3:38:37</t>
         </is>
       </c>
       <c r="I30" t="n">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>F</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1800,7 +1800,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>4小时55分17秒</t>
+          <t>4:55:17</t>
         </is>
       </c>
       <c r="I31" t="n">

</xml_diff>